<commit_message>
chore(gd): 刷新产物 — CodeName 更名 + codename 索引
</commit_message>
<xml_diff>
--- a/gd/excel/ItemType.xlsx
+++ b/gd/excel/ItemType.xlsx
@@ -532,20 +532,71 @@
     <row r="2" ht="38" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Id
-int32</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <color rgb="FF172033"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Id
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <i val="1"/>
+              <color rgb="FF8A5A00"/>
+              <sz val="9"/>
+            </rPr>
+            <t>int32</t>
+          </r>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Name
-string</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <color rgb="FF172033"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Name
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <i val="1"/>
+              <color rgb="FF64748B"/>
+              <sz val="9"/>
+            </rPr>
+            <t>string</t>
+          </r>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Code
-string</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <color rgb="FF172033"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">CodeName
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <i val="1"/>
+              <color rgb="FF64748B"/>
+              <sz val="9"/>
+            </rPr>
+            <t>string</t>
+          </r>
         </is>
       </c>
     </row>

</xml_diff>